<commit_message>
initial push of final files
</commit_message>
<xml_diff>
--- a/Data-paper/1b-reps-10-hypothtest.xlsx
+++ b/Data-paper/1b-reps-10-hypothtest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Research-Published\2021-Baboon FA\BaboonStress\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KaraHoover\Desktop\Hive-local\Projects\baboon-stress\data-paper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A08E8AD7-5B9A-4923-B79C-A885967D865D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C440F457-D3A3-4A23-BD44-EBA5D9A09F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="54060" yWindow="5220" windowWidth="14910" windowHeight="15350" tabRatio="722" xr2:uid="{3123FED7-B888-4F1E-8E92-D9323FB0CFC3}"/>
+    <workbookView xWindow="12960" yWindow="4020" windowWidth="21945" windowHeight="16170" tabRatio="722" xr2:uid="{3123FED7-B888-4F1E-8E92-D9323FB0CFC3}"/>
   </bookViews>
   <sheets>
     <sheet name="FA10" sheetId="10" r:id="rId1"/>
@@ -217,38 +217,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -267,9 +263,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -307,7 +303,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -413,7 +409,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -555,7 +551,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -564,62 +560,60 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B0D2B6B-8F9B-42F5-A6A5-8DA24D60ACED}">
   <dimension ref="A1:P68"/>
-  <sheetFormatPr defaultColWidth="6.5" defaultRowHeight="14.5" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultColWidth="6.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.36328125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.76953125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="6.58984375" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.04296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.6796875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6328125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="6.31640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.31640625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="7.1328125" style="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.31640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5" style="4"/>
-    <col min="13" max="13" width="6.1328125" style="9" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="6.5" style="4"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.140625" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.7">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="6"/>
+      <c r="K1" s="4"/>
       <c r="L1" s="3"/>
-      <c r="M1" s="7"/>
+      <c r="M1" s="5"/>
       <c r="N1" s="3"/>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -647,16 +641,16 @@
       <c r="I2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="11">
+      <c r="J2" s="9">
         <v>6.2767000000000005E-3</v>
       </c>
       <c r="L2" s="2"/>
-      <c r="M2" s="8"/>
+      <c r="M2" s="6"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -684,16 +678,16 @@
       <c r="I3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J3" s="11">
+      <c r="J3" s="9">
         <v>1.15709E-2</v>
       </c>
       <c r="L3" s="2"/>
-      <c r="M3" s="8"/>
+      <c r="M3" s="6"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -721,16 +715,16 @@
       <c r="I4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="9">
         <v>1.0606000000000001E-2</v>
       </c>
       <c r="L4" s="2"/>
-      <c r="M4" s="8"/>
+      <c r="M4" s="6"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -758,16 +752,16 @@
       <c r="I5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="9">
         <v>7.2766999999999997E-3</v>
       </c>
       <c r="L5" s="2"/>
-      <c r="M5" s="8"/>
+      <c r="M5" s="6"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -795,14 +789,14 @@
       <c r="I6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="9">
         <v>2.3969000000000001E-2</v>
       </c>
       <c r="L6" s="2"/>
-      <c r="M6" s="8"/>
+      <c r="M6" s="6"/>
       <c r="N6" s="2"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -830,14 +824,14 @@
       <c r="I7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="9">
         <v>5.0460999999999999E-2</v>
       </c>
       <c r="L7" s="2"/>
-      <c r="M7" s="8"/>
+      <c r="M7" s="6"/>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
@@ -865,13 +859,13 @@
       <c r="I8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="9">
         <v>8.5620000000000002E-3</v>
       </c>
       <c r="L8" s="2"/>
       <c r="N8" s="2"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
@@ -899,13 +893,13 @@
       <c r="I9" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="9">
         <v>2.8579E-2</v>
       </c>
       <c r="L9" s="2"/>
       <c r="N9" s="2"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -933,13 +927,13 @@
       <c r="I10" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="9">
         <v>8.4099999999999991E-3</v>
       </c>
       <c r="L10" s="2"/>
       <c r="N10" s="2"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -967,12 +961,12 @@
       <c r="I11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="9">
         <v>1.7562000000000001E-2</v>
       </c>
       <c r="N11" s="2"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
@@ -1000,12 +994,12 @@
       <c r="I12" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="9">
         <v>3.8048999999999999E-2</v>
       </c>
       <c r="N12" s="2"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>5</v>
       </c>
@@ -1033,12 +1027,12 @@
       <c r="I13" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="9">
         <v>2.8692000000000002E-2</v>
       </c>
       <c r="N13" s="2"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>17</v>
       </c>
@@ -1066,12 +1060,12 @@
       <c r="I14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="9">
         <v>7.5737000000000013E-2</v>
       </c>
       <c r="N14" s="2"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
@@ -1099,12 +1093,12 @@
       <c r="I15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="9">
         <v>7.9821000000000003E-2</v>
       </c>
       <c r="N15" s="2"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.7">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>5</v>
       </c>
@@ -1132,12 +1126,12 @@
       <c r="I16" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="9">
         <v>1.0457000000000001E-2</v>
       </c>
       <c r="N16" s="2"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>5</v>
       </c>
@@ -1165,12 +1159,12 @@
       <c r="I17" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17" s="9">
         <v>4.4386E-3</v>
       </c>
       <c r="N17" s="2"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
@@ -1198,12 +1192,12 @@
       <c r="I18" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="9">
         <v>8.9099999999999995E-3</v>
       </c>
       <c r="N18" s="2"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>5</v>
       </c>
@@ -1231,12 +1225,12 @@
       <c r="I19" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="9">
         <v>3.9489999999999997E-2</v>
       </c>
       <c r="N19" s="2"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>5</v>
       </c>
@@ -1264,13 +1258,13 @@
       <c r="I20" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20" s="9">
         <v>1.3246999999999998E-2</v>
       </c>
       <c r="L20" s="2"/>
       <c r="N20" s="2"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>17</v>
       </c>
@@ -1298,13 +1292,13 @@
       <c r="I21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21" s="9">
         <v>3.0541000000000002E-2</v>
       </c>
       <c r="L21" s="2"/>
       <c r="N21" s="2"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
@@ -1332,13 +1326,13 @@
       <c r="I22" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22" s="9">
         <v>7.9830000000000005E-3</v>
       </c>
       <c r="L22" s="2"/>
       <c r="N22" s="2"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>17</v>
       </c>
@@ -1366,13 +1360,13 @@
       <c r="I23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23" s="9">
         <v>2.0684000000000001E-2</v>
       </c>
       <c r="L23" s="2"/>
       <c r="N23" s="2"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>17</v>
       </c>
@@ -1400,13 +1394,13 @@
       <c r="I24" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J24" s="11">
+      <c r="J24" s="9">
         <v>3.1292E-2</v>
       </c>
       <c r="L24" s="2"/>
       <c r="N24" s="2"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>17</v>
       </c>
@@ -1434,14 +1428,14 @@
       <c r="I25" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25" s="9">
         <v>2.1019000000000003E-2</v>
       </c>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="N25" s="2"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>5</v>
       </c>
@@ -1469,13 +1463,13 @@
       <c r="I26" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J26" s="11">
+      <c r="J26" s="9">
         <v>5.5677999999999991E-2</v>
       </c>
       <c r="K26" s="2"/>
       <c r="N26" s="2"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>5</v>
       </c>
@@ -1503,12 +1497,12 @@
       <c r="I27" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J27" s="9">
         <v>4.3601999999999995E-2</v>
       </c>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>5</v>
       </c>
@@ -1536,12 +1530,12 @@
       <c r="I28" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J28" s="9">
         <v>3.9558999999999997E-2</v>
       </c>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>5</v>
       </c>
@@ -1569,12 +1563,12 @@
       <c r="I29" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29" s="9">
         <v>4.8283E-2</v>
       </c>
       <c r="K29" s="2"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>17</v>
       </c>
@@ -1602,12 +1596,12 @@
       <c r="I30" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30" s="9">
         <v>6.6650000000000001E-2</v>
       </c>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>17</v>
       </c>
@@ -1635,12 +1629,12 @@
       <c r="I31" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J31" s="11">
+      <c r="J31" s="9">
         <v>7.0930999999999994E-2</v>
       </c>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.7">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>17</v>
       </c>
@@ -1668,12 +1662,12 @@
       <c r="I32" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32" s="9">
         <v>9.9453999999999987E-2</v>
       </c>
       <c r="K32" s="2"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
@@ -1681,9 +1675,9 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
-      <c r="J36" s="11"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.7">
+      <c r="J36" s="9"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -1691,9 +1685,9 @@
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
-      <c r="J37" s="11"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.7">
+      <c r="J37" s="9"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -1703,9 +1697,9 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
-      <c r="J38" s="11"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.7">
+      <c r="J38" s="9"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -1715,9 +1709,9 @@
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
-      <c r="J39" s="11"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.7">
+      <c r="J39" s="9"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1727,10 +1721,10 @@
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
-      <c r="J40" s="11"/>
+      <c r="J40" s="9"/>
       <c r="K40" s="2"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1740,10 +1734,10 @@
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
-      <c r="J41" s="11"/>
+      <c r="J41" s="9"/>
       <c r="K41" s="2"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -1755,7 +1749,7 @@
       <c r="I42" s="1"/>
       <c r="K42" s="2"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1767,7 +1761,7 @@
       <c r="I43" s="1"/>
       <c r="K43" s="2"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1779,7 +1773,7 @@
       <c r="I44" s="1"/>
       <c r="K44" s="2"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -1791,7 +1785,7 @@
       <c r="I45" s="1"/>
       <c r="K45" s="2"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1803,7 +1797,7 @@
       <c r="I46" s="1"/>
       <c r="K46" s="2"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1815,7 +1809,7 @@
       <c r="I47" s="1"/>
       <c r="K47" s="2"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -1826,7 +1820,7 @@
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -1837,7 +1831,7 @@
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -1847,9 +1841,9 @@
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
-      <c r="J50" s="11"/>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J50" s="9"/>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -1859,9 +1853,9 @@
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
-      <c r="J51" s="11"/>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J51" s="9"/>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1871,9 +1865,9 @@
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
       <c r="I52" s="1"/>
-      <c r="J52" s="11"/>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J52" s="9"/>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1883,9 +1877,9 @@
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
       <c r="I53" s="1"/>
-      <c r="J53" s="11"/>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J53" s="9"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -1895,9 +1889,9 @@
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
       <c r="I54" s="1"/>
-      <c r="J54" s="11"/>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J54" s="9"/>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -1907,9 +1901,9 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
       <c r="I55" s="1"/>
-      <c r="J55" s="11"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J55" s="9"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -1919,9 +1913,9 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
       <c r="I56" s="1"/>
-      <c r="J56" s="11"/>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J56" s="9"/>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -1931,9 +1925,9 @@
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
       <c r="I57" s="1"/>
-      <c r="J57" s="11"/>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J57" s="9"/>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -1943,9 +1937,9 @@
       <c r="G62" s="1"/>
       <c r="H62" s="1"/>
       <c r="I62" s="1"/>
-      <c r="J62" s="11"/>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J62" s="9"/>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -1955,9 +1949,9 @@
       <c r="G63" s="1"/>
       <c r="H63" s="1"/>
       <c r="I63" s="1"/>
-      <c r="J63" s="11"/>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J63" s="9"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -1967,9 +1961,9 @@
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
       <c r="I64" s="1"/>
-      <c r="J64" s="11"/>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J64" s="9"/>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -1979,9 +1973,9 @@
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="I65" s="1"/>
-      <c r="J65" s="11"/>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J65" s="9"/>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -1991,9 +1985,9 @@
       <c r="G66" s="1"/>
       <c r="H66" s="1"/>
       <c r="I66" s="1"/>
-      <c r="J66" s="11"/>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J66" s="9"/>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -2003,9 +1997,9 @@
       <c r="G67" s="1"/>
       <c r="H67" s="1"/>
       <c r="I67" s="1"/>
-      <c r="J67" s="11"/>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.7">
+      <c r="J67" s="9"/>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -2015,7 +2009,7 @@
       <c r="G68" s="1"/>
       <c r="H68" s="1"/>
       <c r="I68" s="1"/>
-      <c r="J68" s="11"/>
+      <c r="J68" s="9"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J32">

</xml_diff>